<commit_message>
Trazabilidad: Se actualizó el Documento conforme a los cambios realizados en el incremento 3, y de igual forma se actualizó la matríz de RF vs CU acorde a los casos de uso y requerimientos funcionales actuales.
</commit_message>
<xml_diff>
--- a/Documento 0/Matriz_RF_vs_CU .xlsx
+++ b/Documento 0/Matriz_RF_vs_CU .xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="105">
   <si>
     <t>CU1</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>RF51</t>
+  </si>
+  <si>
+    <t>RF52</t>
   </si>
 </sst>
 </file>
@@ -352,7 +355,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -375,12 +378,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFCCCCCC"/>
         <bgColor rgb="FFCCCCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAD3"/>
-        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -435,8 +432,8 @@
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -854,7 +851,9 @@
       <c r="AD2" s="4"/>
       <c r="AE2" s="4"/>
       <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
+      <c r="AG2" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AH2" s="4"/>
       <c r="AI2" s="4"/>
       <c r="AJ2" s="4"/>
@@ -1115,7 +1114,9 @@
       <c r="AG6" s="1"/>
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
-      <c r="AJ6" s="1"/>
+      <c r="AJ6" s="7" t="s">
+        <v>53</v>
+      </c>
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
       <c r="AM6" s="1"/>
@@ -1370,7 +1371,9 @@
       <c r="AD10" s="1"/>
       <c r="AE10" s="1"/>
       <c r="AF10" s="1"/>
-      <c r="AG10" s="1"/>
+      <c r="AG10" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AH10" s="1"/>
       <c r="AI10" s="1"/>
       <c r="AJ10" s="1"/>
@@ -1429,7 +1432,9 @@
       <c r="AD11" s="1"/>
       <c r="AE11" s="1"/>
       <c r="AF11" s="1"/>
-      <c r="AG11" s="1"/>
+      <c r="AG11" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AH11" s="1"/>
       <c r="AI11" s="1"/>
       <c r="AJ11" s="1"/>
@@ -2002,9 +2007,7 @@
       <c r="AF20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AG20" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AG20" s="1"/>
       <c r="AH20" s="1"/>
       <c r="AI20" s="1"/>
       <c r="AJ20" s="1"/>
@@ -2208,7 +2211,7 @@
       <c r="BA23" s="1"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B24" s="6"/>
@@ -2258,9 +2261,7 @@
       <c r="AT24" s="1"/>
       <c r="AU24" s="1"/>
       <c r="AV24" s="1"/>
-      <c r="AW24" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AW24" s="1"/>
       <c r="AX24" s="1"/>
       <c r="AY24" s="1"/>
       <c r="AZ24" s="1"/>
@@ -2311,7 +2312,9 @@
       <c r="AJ25" s="1"/>
       <c r="AK25" s="1"/>
       <c r="AL25" s="1"/>
-      <c r="AM25" s="1"/>
+      <c r="AM25" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AN25" s="1"/>
       <c r="AO25" s="1"/>
       <c r="AP25" s="1"/>
@@ -2321,7 +2324,9 @@
       <c r="AT25" s="1"/>
       <c r="AU25" s="1"/>
       <c r="AV25" s="1"/>
-      <c r="AW25" s="1"/>
+      <c r="AW25" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AX25" s="1"/>
       <c r="AY25" s="1"/>
       <c r="AZ25" s="1"/>
@@ -2380,9 +2385,7 @@
       <c r="AT26" s="1"/>
       <c r="AU26" s="1"/>
       <c r="AV26" s="1"/>
-      <c r="AW26" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AW26" s="1"/>
       <c r="AX26" s="1"/>
       <c r="AY26" s="1"/>
       <c r="AZ26" s="1"/>
@@ -2669,9 +2672,7 @@
       <c r="AF31" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AG31" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AG31" s="1"/>
       <c r="AH31" s="1"/>
       <c r="AI31" s="1"/>
       <c r="AJ31" s="1"/>
@@ -2728,9 +2729,7 @@
       <c r="AD32" s="1"/>
       <c r="AE32" s="1"/>
       <c r="AF32" s="1"/>
-      <c r="AG32" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AG32" s="1"/>
       <c r="AH32" s="1"/>
       <c r="AI32" s="1"/>
       <c r="AJ32" s="1"/>
@@ -2743,7 +2742,9 @@
       <c r="AQ32" s="1"/>
       <c r="AR32" s="1"/>
       <c r="AS32" s="1"/>
-      <c r="AT32" s="1"/>
+      <c r="AT32" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AU32" s="1"/>
       <c r="AV32" s="1"/>
       <c r="AW32" s="1"/>
@@ -2910,14 +2911,10 @@
       <c r="AG35" s="1"/>
       <c r="AH35" s="1"/>
       <c r="AI35" s="1"/>
-      <c r="AJ35" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AJ35" s="1"/>
       <c r="AK35" s="1"/>
       <c r="AL35" s="1"/>
-      <c r="AM35" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AM35" s="1"/>
       <c r="AN35" s="1"/>
       <c r="AO35" s="1"/>
       <c r="AP35" s="1"/>
@@ -2929,7 +2926,9 @@
       <c r="AV35" s="1"/>
       <c r="AW35" s="1"/>
       <c r="AX35" s="1"/>
-      <c r="AY35" s="1"/>
+      <c r="AY35" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AZ35" s="1"/>
       <c r="BA35" s="1"/>
     </row>
@@ -3098,9 +3097,7 @@
       <c r="AJ38" s="1"/>
       <c r="AK38" s="1"/>
       <c r="AL38" s="1"/>
-      <c r="AM38" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AM38" s="1"/>
       <c r="AN38" s="1"/>
       <c r="AO38" s="1"/>
       <c r="AP38" s="1"/>
@@ -3777,9 +3774,7 @@
       <c r="AT49" s="1"/>
       <c r="AU49" s="1"/>
       <c r="AV49" s="1"/>
-      <c r="AW49" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AW49" s="1"/>
       <c r="AX49" s="1"/>
       <c r="AY49" s="1"/>
       <c r="AZ49" s="1"/>
@@ -3884,7 +3879,9 @@
       <c r="AG51" s="1"/>
       <c r="AH51" s="1"/>
       <c r="AI51" s="1"/>
-      <c r="AJ51" s="1"/>
+      <c r="AJ51" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="AK51" s="1"/>
       <c r="AL51" s="1"/>
       <c r="AM51" s="1"/>
@@ -3899,9 +3896,7 @@
       <c r="AV51" s="1"/>
       <c r="AW51" s="1"/>
       <c r="AX51" s="1"/>
-      <c r="AY51" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="AY51" s="1"/>
       <c r="AZ51" s="1"/>
       <c r="BA51" s="1"/>
     </row>
@@ -3966,7 +3961,67 @@
       </c>
       <c r="BA52" s="1"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+      <c r="N53" s="1"/>
+      <c r="O53" s="1"/>
+      <c r="P53" s="1"/>
+      <c r="Q53" s="1"/>
+      <c r="R53" s="1"/>
+      <c r="S53" s="1"/>
+      <c r="T53" s="1"/>
+      <c r="U53" s="1"/>
+      <c r="V53" s="1"/>
+      <c r="W53" s="1"/>
+      <c r="X53" s="1"/>
+      <c r="Y53" s="1"/>
+      <c r="Z53" s="1"/>
+      <c r="AA53" s="1"/>
+      <c r="AB53" s="1"/>
+      <c r="AC53" s="1"/>
+      <c r="AD53" s="1"/>
+      <c r="AE53" s="1"/>
+      <c r="AF53" s="1"/>
+      <c r="AG53" s="1"/>
+      <c r="AH53" s="1"/>
+      <c r="AI53" s="1"/>
+      <c r="AJ53" s="1"/>
+      <c r="AK53" s="1"/>
+      <c r="AL53" s="1"/>
+      <c r="AM53" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN53" s="1"/>
+      <c r="AO53" s="1"/>
+      <c r="AP53" s="1"/>
+      <c r="AQ53" s="1"/>
+      <c r="AR53" s="1"/>
+      <c r="AS53" s="1"/>
+      <c r="AT53" s="1"/>
+      <c r="AU53" s="1"/>
+      <c r="AV53" s="1"/>
+      <c r="AW53" s="1"/>
+      <c r="AX53" s="1"/>
+      <c r="AY53" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AZ53" s="1"/>
+      <c r="BA53" s="1"/>
+    </row>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>

</xml_diff>